<commit_message>
Pantalla Nueva Venta Renta Fija rediseño con campos autocalculados
</commit_message>
<xml_diff>
--- a/documentacion/EjemploVenta.xlsx
+++ b/documentacion/EjemploVenta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40950C3E-43EF-4F25-9A6D-798918B46BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A156FB1-B823-4BDA-BD5F-CFE7FAF8D5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{61F106E6-B575-4EC4-BC00-461AB029E228}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{61F106E6-B575-4EC4-BC00-461AB029E228}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Se corrigen calculos relacionados con la venta de inversiones de rentabilidad fija
</commit_message>
<xml_diff>
--- a/documentacion/EjemploVenta.xlsx
+++ b/documentacion/EjemploVenta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A156FB1-B823-4BDA-BD5F-CFE7FAF8D5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB68DD0D-E014-458E-9C0A-05EC19B15F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{61F106E6-B575-4EC4-BC00-461AB029E228}"/>
   </bookViews>
@@ -303,7 +303,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -340,6 +340,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="16">
     <border>
@@ -549,7 +555,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -584,7 +590,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="4" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -626,6 +631,11 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -998,66 +1008,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4617800B-0C8A-4C80-8ADE-43650974D16B}">
-  <dimension ref="A1:AQ5"/>
+  <dimension ref="A1:AQ18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="15.7109375" customWidth="1"/>
     <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="19" max="20" width="11.42578125" style="13"/>
-    <col min="29" max="29" width="11.42578125" style="13"/>
+    <col min="19" max="20" width="11.85546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.85546875" style="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="37"/>
-      <c r="R1" s="37"/>
-      <c r="S1" s="37"/>
-      <c r="T1" s="37"/>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="37"/>
-      <c r="X1" s="37"/>
-      <c r="Y1" s="37"/>
-      <c r="Z1" s="37"/>
-      <c r="AA1" s="37"/>
-      <c r="AB1" s="38"/>
-      <c r="AC1" s="33" t="s">
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+      <c r="P1" s="36"/>
+      <c r="Q1" s="36"/>
+      <c r="R1" s="36"/>
+      <c r="S1" s="36"/>
+      <c r="T1" s="36"/>
+      <c r="U1" s="36"/>
+      <c r="V1" s="36"/>
+      <c r="W1" s="36"/>
+      <c r="X1" s="36"/>
+      <c r="Y1" s="36"/>
+      <c r="Z1" s="36"/>
+      <c r="AA1" s="36"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="AD1" s="34"/>
-      <c r="AE1" s="34"/>
-      <c r="AF1" s="34"/>
-      <c r="AG1" s="34"/>
-      <c r="AH1" s="34"/>
-      <c r="AI1" s="34"/>
-      <c r="AJ1" s="34"/>
-      <c r="AK1" s="34"/>
-      <c r="AL1" s="34"/>
-      <c r="AM1" s="34"/>
-      <c r="AN1" s="34"/>
-      <c r="AO1" s="34"/>
-      <c r="AP1" s="34"/>
-      <c r="AQ1" s="35"/>
+      <c r="AD1" s="33"/>
+      <c r="AE1" s="33"/>
+      <c r="AF1" s="33"/>
+      <c r="AG1" s="33"/>
+      <c r="AH1" s="33"/>
+      <c r="AI1" s="33"/>
+      <c r="AJ1" s="33"/>
+      <c r="AK1" s="33"/>
+      <c r="AL1" s="33"/>
+      <c r="AM1" s="33"/>
+      <c r="AN1" s="33"/>
+      <c r="AO1" s="33"/>
+      <c r="AP1" s="33"/>
+      <c r="AQ1" s="34"/>
     </row>
     <row r="2" spans="1:43" s="1" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1066,79 +1076,79 @@
       <c r="C2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="29" t="s">
+      <c r="F2" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="29" t="s">
+      <c r="G2" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="29" t="s">
+      <c r="H2" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="29" t="s">
+      <c r="I2" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="29" t="s">
+      <c r="J2" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="29" t="s">
+      <c r="K2" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="29" t="s">
+      <c r="L2" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="M2" s="29" t="s">
+      <c r="M2" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="N2" s="29" t="s">
+      <c r="N2" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="29" t="s">
+      <c r="O2" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="29" t="s">
+      <c r="P2" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="Q2" s="30" t="s">
+      <c r="Q2" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="R2" s="30" t="s">
+      <c r="R2" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="31" t="s">
+      <c r="S2" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="T2" s="31" t="s">
+      <c r="T2" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="29" t="s">
+      <c r="U2" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="30" t="s">
+      <c r="V2" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="W2" s="30" t="s">
+      <c r="W2" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="X2" s="30" t="s">
+      <c r="X2" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="Y2" s="30" t="s">
+      <c r="Y2" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="Z2" s="30" t="s">
+      <c r="Z2" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="AA2" s="30" t="s">
+      <c r="AA2" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="AB2" s="32" t="s">
+      <c r="AB2" s="31" t="s">
         <v>25</v>
       </c>
       <c r="AC2" s="20" t="s">
@@ -1277,37 +1287,37 @@
         <v>18.18</v>
       </c>
       <c r="AB3" s="18"/>
-      <c r="AC3" s="22">
+      <c r="AC3" s="38">
         <v>89.245310000000003</v>
       </c>
       <c r="AD3" s="8"/>
-      <c r="AE3" s="9">
+      <c r="AE3" s="39">
         <v>27.898661338661341</v>
       </c>
-      <c r="AF3" s="9">
+      <c r="AF3" s="39">
         <f t="shared" ref="AF3" si="9">AC3*R3/100</f>
         <v>6193.6245140000001</v>
       </c>
-      <c r="AG3" s="9">
+      <c r="AG3" s="39">
         <v>61.93308691308691</v>
       </c>
-      <c r="AH3" s="9">
+      <c r="AH3" s="39">
         <v>3.0990809190809192</v>
       </c>
-      <c r="AI3" s="9">
+      <c r="AI3" s="39">
         <f t="shared" ref="AI3:AI4" si="10">AF3-AG3-AH3</f>
         <v>6128.5923461678321</v>
       </c>
-      <c r="AJ3" s="9">
-        <f t="shared" ref="AJ3:AJ4" si="11">AF3-U3</f>
+      <c r="AJ3" s="39">
+        <f>AF3-U3</f>
         <v>1353.6102783780007</v>
       </c>
-      <c r="AK3" s="9">
-        <f t="shared" ref="AK3:AK4" si="12">AI3-V3</f>
+      <c r="AK3" s="39">
+        <f t="shared" ref="AK3:AK4" si="11">AI3-V3</f>
         <v>1270.3981105458333</v>
       </c>
       <c r="AL3" s="9">
-        <f t="shared" ref="AL3:AL4" si="13">AK3+Q3+AE3</f>
+        <f t="shared" ref="AL3:AL4" si="12">AK3+Q3+AE3</f>
         <v>1845.942771884495</v>
       </c>
       <c r="AM3" s="10">
@@ -1315,18 +1325,18 @@
         <v>534</v>
       </c>
       <c r="AN3" s="11">
-        <f t="shared" ref="AN3:AN4" si="14">AL3/V3</f>
+        <f t="shared" ref="AN3:AN4" si="13">AL3/V3</f>
         <v>0.37996479398649596</v>
       </c>
       <c r="AO3" s="11">
-        <f t="shared" ref="AO3:AO4" si="15">AL3/V3*365/AM3</f>
+        <f t="shared" ref="AO3:AO4" si="14">AL3/V3*365/AM3</f>
         <v>0.25971376367990828</v>
       </c>
       <c r="AP3" s="11">
-        <f t="shared" ref="AP3:AP4" si="16">POWER((1+AN3),(365/AM3))-1</f>
+        <f t="shared" ref="AP3:AP4" si="15">POWER((1+AN3),(365/AM3))-1</f>
         <v>0.24624280434490431</v>
       </c>
-      <c r="AQ3" s="23" t="e">
+      <c r="AQ3" s="22" t="e">
         <f>[1]!TitulosVendidos[[#This Row],[Comisión Santa Fe
 Venta]]+[1]!TitulosVendidos[[#This Row],[Comisión Santa Fé
 Compra]]</f>
@@ -1423,37 +1433,37 @@
         <v>14</v>
       </c>
       <c r="AB4" s="18"/>
-      <c r="AC4" s="22">
+      <c r="AC4" s="38">
         <v>89.245310000000003</v>
       </c>
       <c r="AD4" s="8"/>
-      <c r="AE4" s="9">
+      <c r="AE4" s="39">
         <v>12.341338661338662</v>
       </c>
-      <c r="AF4" s="9">
+      <c r="AF4" s="39">
         <f>AC4*R4/100</f>
         <v>2739.831017</v>
       </c>
-      <c r="AG4" s="9">
+      <c r="AG4" s="39">
         <v>27.396913086913084</v>
       </c>
-      <c r="AH4" s="9">
+      <c r="AH4" s="39">
         <v>1.370919080919081</v>
       </c>
-      <c r="AI4" s="9">
+      <c r="AI4" s="39">
         <f t="shared" si="10"/>
         <v>2711.0631848321677</v>
       </c>
-      <c r="AJ4" s="9">
+      <c r="AJ4" s="39">
+        <f t="shared" ref="AJ3:AJ4" si="16">AF4-U4</f>
+        <v>597.80109618699998</v>
+      </c>
+      <c r="AK4" s="39">
         <f t="shared" si="11"/>
-        <v>597.80109618699998</v>
-      </c>
-      <c r="AK4" s="9">
+        <v>555.03326401916729</v>
+      </c>
+      <c r="AL4" s="9">
         <f t="shared" si="12"/>
-        <v>555.03326401916729</v>
-      </c>
-      <c r="AL4" s="9">
-        <f t="shared" si="13"/>
         <v>808.26260268050601</v>
       </c>
       <c r="AM4" s="10">
@@ -1461,18 +1471,18 @@
         <v>531</v>
       </c>
       <c r="AN4" s="11">
+        <f t="shared" si="13"/>
+        <v>0.37488468730328406</v>
+      </c>
+      <c r="AO4" s="11">
         <f t="shared" si="14"/>
-        <v>0.37488468730328406</v>
-      </c>
-      <c r="AO4" s="11">
+        <v>0.25768909767551545</v>
+      </c>
+      <c r="AP4" s="11">
         <f t="shared" si="15"/>
-        <v>0.25768909767551545</v>
-      </c>
-      <c r="AP4" s="11">
-        <f t="shared" si="16"/>
         <v>0.24463437049247494</v>
       </c>
-      <c r="AQ4" s="23" t="e">
+      <c r="AQ4" s="22" t="e">
         <f>[1]!TitulosVendidos[[#This Row],[Comisión Santa Fe
 Venta]]+[1]!TitulosVendidos[[#This Row],[Comisión Santa Fé
 Compra]]</f>
@@ -1514,31 +1524,108 @@
       <c r="Z5" s="15"/>
       <c r="AA5" s="15"/>
       <c r="AB5" s="19"/>
-      <c r="AC5" s="24" t="s">
+      <c r="AC5" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="AD5" s="25"/>
-      <c r="AE5" s="26" t="s">
+      <c r="AD5" s="24"/>
+      <c r="AE5" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="AF5" s="26"/>
-      <c r="AG5" s="26" t="s">
+      <c r="AF5" s="25"/>
+      <c r="AG5" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="AH5" s="26" t="s">
+      <c r="AH5" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="AI5" s="26" t="s">
+      <c r="AI5" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="AJ5" s="25"/>
-      <c r="AK5" s="25"/>
-      <c r="AL5" s="25"/>
-      <c r="AM5" s="25"/>
-      <c r="AN5" s="25"/>
-      <c r="AO5" s="25"/>
-      <c r="AP5" s="25"/>
-      <c r="AQ5" s="27"/>
+      <c r="AJ5" s="24"/>
+      <c r="AK5" s="24"/>
+      <c r="AL5" s="24"/>
+      <c r="AM5" s="24"/>
+      <c r="AN5" s="24"/>
+      <c r="AO5" s="24"/>
+      <c r="AP5" s="24"/>
+      <c r="AQ5" s="26"/>
+    </row>
+    <row r="9" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AI9">
+        <v>6156.49</v>
+      </c>
+      <c r="AL9" s="40">
+        <v>6193.62</v>
+      </c>
+      <c r="AO9">
+        <v>794.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AI10">
+        <v>2723.4</v>
+      </c>
+      <c r="AL10" s="40"/>
+      <c r="AO10">
+        <v>13.712666666666669</v>
+      </c>
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AE11">
+        <v>227.13</v>
+      </c>
+      <c r="AI11">
+        <f>SUM(AI9:AI10)</f>
+        <v>8879.89</v>
+      </c>
+      <c r="AL11" s="40">
+        <v>61.93</v>
+      </c>
+      <c r="AO11">
+        <f>AO9+AO10</f>
+        <v>808.21266666666668</v>
+      </c>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AE12">
+        <v>555.03326401916729</v>
+      </c>
+      <c r="AL12" s="40">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AE13" s="39">
+        <v>12.341338661338662</v>
+      </c>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AE14">
+        <f>SUM(AE11:AE13)</f>
+        <v>794.50460268050597</v>
+      </c>
+    </row>
+    <row r="15" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AL15">
+        <f>AL9+AL10-AL11-AL12</f>
+        <v>6128.5899999999992</v>
+      </c>
+    </row>
+    <row r="16" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AG16">
+        <v>6156.49</v>
+      </c>
+    </row>
+    <row r="17" spans="33:33" x14ac:dyDescent="0.25">
+      <c r="AG17">
+        <v>2723.4</v>
+      </c>
+    </row>
+    <row r="18" spans="33:33" x14ac:dyDescent="0.25">
+      <c r="AG18">
+        <f>SUM(AG16:AG17)</f>
+        <v>8879.89</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>